<commit_message>
Mejora visual finanzas públicas
</commit_message>
<xml_diff>
--- a/data/raw/sistema_alertas.xlsx
+++ b/data/raw/sistema_alertas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e_edobru\Desktop\Bancomext\Estatales\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C16A281-8867-4C2D-8F88-0249F5CA9D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D3C2D6-E988-4B77-9780-B399343E1739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-6855" windowWidth="29040" windowHeight="15720" xr2:uid="{9566E5A0-6D86-410A-B775-C39A22568F0C}"/>
   </bookViews>
@@ -739,6 +739,8 @@
       <c r="E2">
         <v>5.0000000000000001E-3</v>
       </c>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">

</xml_diff>